<commit_message>
updated Script 5 to match new analysis, checked by Cole
</commit_message>
<xml_diff>
--- a/outputs/step_outputs/05_figure_did_summary.xlsx
+++ b/outputs/step_outputs/05_figure_did_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,27 +441,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>real_did_injury_200m</t>
+          <t>real_did_injury</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>placebo_did_injury_200m</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>did_injury_150m</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>did_injury_200m</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>did_injury_250m</t>
+          <t>placebo_did_injury</t>
         </is>
       </c>
     </row>
@@ -478,16 +463,7 @@
         <v>-17.29</v>
       </c>
       <c r="D2" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-6.69</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-17.29</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-8.57</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="3">
@@ -500,19 +476,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>-14.26</v>
+        <v>-15.8</v>
       </c>
       <c r="D3" t="n">
         <v>-17.01</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-29.55</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-14.26</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-13.01</v>
       </c>
     </row>
     <row r="4">
@@ -525,19 +492,10 @@
         <v>56</v>
       </c>
       <c r="C4" t="n">
-        <v>2.14</v>
+        <v>2.27</v>
       </c>
       <c r="D4" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.68</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="5">
@@ -553,16 +511,7 @@
         <v>6.66</v>
       </c>
       <c r="D5" t="n">
-        <v>-7.53</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6.46</v>
-      </c>
-      <c r="F5" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="G5" t="n">
-        <v>6.87</v>
+        <v>-7.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>